<commit_message>
publish: 4ccfe136c036c49e0700d35d391c63dc9c8cc8e7 (run 32551602944)
</commit_message>
<xml_diff>
--- a/CodeSystem-CS-BetelNutComponent.xlsx
+++ b/CodeSystem-CS-BetelNutComponent.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-22T02:14:01+00:00</t>
+    <t>2026-08-22T04:25:10+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -147,7 +147,7 @@
     <t>每日嚼食量</t>
   </si>
   <si>
-    <t>每日嚼食檳榔之顆數，以 UCUM 單位「{quid}/d」表達。承載主管機關最小上傳集第 10 列（醫令 30907X-2「嚼檳量」）。⚠️ 原案該列為複合欄位，同時收「平均每日嚼幾顆」與「嚼檳年數」兩個量綱不同之值，於資料交換時難以拆解；經本案專家會議［專家會議場次與日期待補］決議，年數移列第 11 列，本欄僅承載每日顆數。單位原案記「{個}/d」，惟 UCUM 之 annotation 僅接受可列印 ASCII，「{個}」非合法 UCUM，故採「{quid}/d」——此為術語技術正確性之更正，不涉語意，數值意義完全相同。本項屬受託團隊職權範圍之技術決議，無須委託單位或主管機關另行核定。對應上游 sf-BetNutChewBeh#amount。</t>
+    <t>每日嚼食檳榔之顆數，以 UCUM 單位「{quid}/d」表達。承載主管機關最小上傳集第 10 列（醫令 30907X-2「嚼檳量」）。⚠️ 原案該列為複合欄位，同時收「平均每日嚼幾顆」與「嚼檳年數」兩個量綱不同之值，於資料交換時難以拆解；本欄僅承載每日顆數，年數移列第 11 列——第 11 列之語意經本案專家共識會議（2026-07-17）七、臨時動議決議更正為嚼食持續期間，年數乃隨之移列。單位原案記「{個}/d」，惟 UCUM 之 annotation 僅接受可列印 ASCII，「{個}」非合法 UCUM，故採「{quid}/d」——此為術語技術正確性之更正，不涉語意，數值意義完全相同。本項屬受託團隊職權範圍之技術決議，無須委託單位或主管機關另行核定。對應上游 sf-BetNutChewBeh#amount。</t>
   </si>
   <si>
     <t>duration-years</t>
@@ -156,7 +156,7 @@
     <t>嚼食持續期間</t>
   </si>
   <si>
-    <t>嚼食檳榔之持續期間（嚼了多久），以 UCUM 單位「a」或「mo」表達，並以原始採集粒度為準——不得將「嚼 2 年」逕行改寫為 24 個月。承載主管機關最小上傳集第 11 列（醫令 30907X-3，原案欄名「嚼檳月數」）。⚠️ 本欄不論受檢者現仍嚼食或已戒除，均應填列——嚼食持續期間是檳榔相關口腔癌之核心累積暴露指標，不因戒除而消失。戒除資訊另由 cessationDuration（戒除期間）與 cessationDate（戒除日期）承載，不佔上傳集之列位。原案該列之 r4 值規則寫「填寫戒檳月數」，經本案專家會議［專家會議場次與日期待補］指出係原案文字有誤並決議更正為嚼食持續期間；本項屬受託團隊職權範圍之技術決議，無須委託單位或主管機關另行核定。對應上游 sf-BetNutChewBeh#year。⚠️ 代碼 id 保留「duration-years」係因該碼已於 v0.4.0 發佈，改名屬破壞性變更；真實語意以本顯示名與定義為準。</t>
+    <t>嚼食檳榔之持續期間（嚼了多久），以 UCUM 單位「a」或「mo」表達，並以原始採集粒度為準——不得將「嚼 2 年」逕行改寫為 24 個月。承載主管機關最小上傳集第 11 列（醫令 30907X-3，原案欄名「嚼檳月數」）。⚠️ 本欄不論受檢者現仍嚼食或已戒除，均應填列——嚼食持續期間是檳榔相關口腔癌之核心累積暴露指標，不因戒除而消失。戒除資訊另由 cessationDuration（戒除期間）與 cessationDate（戒除日期）承載，不佔上傳集之列位。原案該列之 r4 值規則寫「填寫戒檳月數」，經本案專家共識會議（臺灣勞工健康檢查核心資料集與 FHIR IG 專家共識討論會，2026-07-17）七、臨時動議認定係原案文字有誤，決議更正為嚼食持續期間，且不論現嚼或已戒均應填列；共同主持人曹又中主任（職業醫學科）另於 2026-07-31 回信補充說明；本項屬受託團隊職權範圍之技術決議，無須委託單位或主管機關另行核定。對應上游 sf-BetNutChewBeh#year。⚠️ 代碼 id 保留「duration-years」係因該碼已於 v0.4.0 發佈，改名屬破壞性變更；真實語意以本顯示名與定義為準。</t>
   </si>
   <si>
     <t>cessation-duration</t>
@@ -165,7 +165,7 @@
     <t>戒除期間</t>
   </si>
   <si>
-    <t>已戒除之期間，以 UCUM 單位「a」或「mo」表達，並以原始採集粒度為準——不得將「已戒 1 年」逕行改寫為 12 個月。⚠️ 本欄與 cessationDate 共同承接主管機關原案第 11 列 r4 所指之「戒檳月數」：該列語意經本案專家會議決議更正為嚼食持續期間後，戒除資訊改由本欄承載，不佔上傳集之列位。故本次語意更正並不造成任何資訊遺失。對應上游 sf-BetNutChewBeh#quit。</t>
+    <t>已戒除之期間，以 UCUM 單位「a」或「mo」表達，並以原始採集粒度為準——不得將「已戒 1 年」逕行改寫為 12 個月。⚠️ 本欄與 cessationDate 共同承接主管機關原案第 11 列 r4 所指之「戒檳月數」：該列語意經本案專家共識會議（2026-07-17）決議更正為嚼食持續期間後，戒除資訊改由本欄承載，不佔上傳集之列位。故本次語意更正並不造成任何資訊遺失。對應上游 sf-BetNutChewBeh#quit。</t>
   </si>
   <si>
     <t>cessation-date</t>

</xml_diff>